<commit_message>
updated code for Hungary
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Belgium_Regression_PK17.xlsx
+++ b/Data/Hires/Workday_NewHire_Belgium_Regression_PK17.xlsx
@@ -1,34 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A1B813-C4A2-43D8-9B8A-77E97390D98D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7360"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="131">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -228,6 +214,12 @@
     <t>Test1</t>
   </si>
   <si>
+    <t>10699085</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
     <t>751 Retail Team 1 (Rykec Puvyjo (10528834) (Inherited))</t>
   </si>
   <si>
@@ -237,10 +229,10 @@
     <t>Mr</t>
   </si>
   <si>
-    <t>Tyson</t>
-  </si>
-  <si>
-    <t>Block</t>
+    <t>Alfred</t>
+  </si>
+  <si>
+    <t>Torphy</t>
   </si>
   <si>
     <t>Landline</t>
@@ -372,19 +364,22 @@
     <t>Test2</t>
   </si>
   <si>
+    <t>10699086</t>
+  </si>
+  <si>
     <t>751 Store Management (Rykec Puvyjo (10528834))</t>
   </si>
   <si>
     <t>Mme</t>
   </si>
   <si>
-    <t>Betty</t>
-  </si>
-  <si>
-    <t>Wilderman</t>
-  </si>
-  <si>
-    <t>Auto 78210614</t>
+    <t>Teresa</t>
+  </si>
+  <si>
+    <t>Mayer</t>
+  </si>
+  <si>
+    <t>Auto 78716171</t>
   </si>
   <si>
     <t>Fixed Term (Fixed Term)</t>
@@ -417,58 +412,58 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color indexed="8"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color indexed="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FF4A4A4A"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color rgb="FF1F1F1F"/>
+      <family val="3"/>
       <sz val="6"/>
-      <color rgb="FF1F1F1F"/>
       <name val="Courier New"/>
-      <family val="3"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FF800000"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="6">
@@ -480,19 +475,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.1499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -517,12 +512,8 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -532,25 +523,15 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -561,22 +542,14 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
+      <left style="thin"/>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -970,9 +943,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BP3"/>
-  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
@@ -1041,7 +1014,7 @@
     <col min="68" max="68" width="16.54296875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.5" customHeight="1" spans="1:68" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1247,45 +1220,49 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="12"/>
+      <c r="B2" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>67</v>
+      </c>
       <c r="D2" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G2" s="16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I2" s="18">
         <v>25041111</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K2" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L2" s="19">
-        <f t="shared" ref="L2" ca="1" si="0">TODAY()-31</f>
+        <f t="shared" ref="L2" si="0">TODAY()-31</f>
         <v>45761</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N2" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O2" s="18">
         <v>38</v>
@@ -1294,44 +1271,44 @@
         <v>1000</v>
       </c>
       <c r="Q2" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="R2" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="S2" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="R2" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="S2" s="18" t="s">
-        <v>72</v>
-      </c>
       <c r="T2" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="U2" s="22" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="V2" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="W2" s="23">
-        <f t="shared" ref="W2" ca="1" si="1">L2</f>
+        <f t="shared" ref="W2" si="1">L2</f>
         <v>45761</v>
       </c>
       <c r="X2" s="18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="Y2" s="24" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="Z2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AA2" s="25" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="AB2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC2" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AD2" s="1" t="s">
         <v>52</v>
@@ -1340,157 +1317,162 @@
         <v>35</v>
       </c>
       <c r="AF2" s="27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AG2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AH2" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AI2" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AJ2" s="18" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AK2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="AL2" s="28" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AM2" s="28" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AN2" s="1">
-        <f t="array" aca="1" ref="AN2:AN3" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
+        <f t="array" ref="AN2:AN3">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
         <v>17338930760</v>
       </c>
       <c r="AO2" s="14" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AP2" s="20" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AQ2" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="AR2" s="19" t="str">
+        <v>95</v>
+      </c>
+      <c r="AR2" s="19">
         <f>AH2</f>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AS2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AT2" s="29">
         <v>35591</v>
       </c>
       <c r="AU2" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="AV2" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW2" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="AX2" s="30" t="s">
+        <v>97</v>
+      </c>
+      <c r="AY2" s="31" t="s">
+        <v>98</v>
+      </c>
+      <c r="AZ2" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="BA2" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>100</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>101</v>
+      </c>
+      <c r="BD2" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="BE2" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="BF2" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="BG2" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="BH2" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="BI2" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="BJ2" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="BK2" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="BL2" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="BM2" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="BN2" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="BO2" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="BP2" s="33" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="AV2" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="AW2" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="AX2" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="AY2" s="31" t="s">
-        <v>96</v>
-      </c>
-      <c r="AZ2" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="BA2" s="30" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB2" t="s">
-        <v>98</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>99</v>
-      </c>
-      <c r="BD2" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="BE2" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="BF2" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="BG2" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="BH2" s="28" t="s">
-        <v>104</v>
-      </c>
-      <c r="BI2" s="28" t="s">
-        <v>105</v>
-      </c>
-      <c r="BJ2" s="30" t="s">
-        <v>106</v>
-      </c>
-      <c r="BK2" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="BL2" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="BM2" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="BN2" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="BO2" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="BP2" s="33" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C3" s="12"/>
       <c r="D3" s="13" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="I3" s="18">
         <v>25041111</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K3" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L3" s="19">
-        <f t="shared" ref="L3" ca="1" si="2">TODAY()-31</f>
+        <f t="shared" ref="L3" si="2">TODAY()-31</f>
         <v>45761</v>
       </c>
       <c r="M3" s="14" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N3" s="20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O3" s="18">
         <v>38</v>
@@ -1499,44 +1481,44 @@
         <v>1000</v>
       </c>
       <c r="Q3" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="R3" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="S3" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="R3" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="S3" s="18" t="s">
-        <v>72</v>
-      </c>
       <c r="T3" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="U3" s="22" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="V3" s="18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="W3" s="23">
-        <f t="shared" ref="W3" ca="1" si="3">L3</f>
+        <f t="shared" ref="W3" si="3">L3</f>
         <v>45761</v>
       </c>
       <c r="X3" s="18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="Y3" s="24" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="Z3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="AA3" s="25" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="AB3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="AC3" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>52</v>
@@ -1545,132 +1527,149 @@
         <v>35</v>
       </c>
       <c r="AF3" s="14" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="AG3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="AH3" s="19">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46157</v>
       </c>
       <c r="AI3" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="AJ3" s="18" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="AK3" s="1">
         <v>251</v>
       </c>
       <c r="AL3" s="28" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AM3" s="28" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AN3" s="1">
-        <f ca="1"/>
         <v>32286014594</v>
       </c>
       <c r="AO3" s="14" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AP3" s="20" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="AQ3" s="20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AR3" s="19">
-        <f t="shared" ref="AR3" ca="1" si="4">AH3</f>
+        <f t="shared" ref="AR3" si="4">AH3</f>
         <v>46157</v>
       </c>
       <c r="AS3" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="AT3" s="29">
         <v>35591</v>
       </c>
       <c r="AU3" s="30" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AV3" s="28" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="AW3" s="30" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="AX3" s="30" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AY3" s="31" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AZ3" s="30" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="BA3" s="30" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="BB3" s="34" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="BC3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="BD3" s="14" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="BE3" s="28" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="BF3" s="32" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="BG3" s="28" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="BH3" s="28" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BI3" s="28" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="BJ3" s="30" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="BK3" s="30" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="BL3" s="30" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BM3" s="30" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BN3" s="30" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BO3" s="18" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BP3" s="33" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ3 X2:X3 V2:V3 S2:S3 K2:K3 BI2:BI3 AX2:AX3" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="7">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ3">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX3">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2:BI3">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K3">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S3">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V3">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X3">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="U3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="U2" r:id="rId1"/>
+    <hyperlink ref="U3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Web Action pages maintaned.
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Belgium_Regression_PK17.xlsx
+++ b/Data/Hires/Workday_NewHire_Belgium_Regression_PK17.xlsx
@@ -1,20 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10245CC-9467-469D-9D09-9E9CEB96C8FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="128">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -214,12 +228,6 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10699755</t>
-  </si>
-  <si>
-    <t>Passed</t>
-  </si>
-  <si>
     <t>751 Retail Team 1 (Rykec Puvyjo (10528834) (Inherited))</t>
   </si>
   <si>
@@ -362,15 +370,6 @@
   </si>
   <si>
     <t>Test2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test failed for 'Cristina Heidenreich' Employee:{10699776}TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for getByRole('button', { name: 'Hire: Cristina Heidenreich' }).first()[22m
-</t>
-  </si>
-  <si>
-    <t>Failed</t>
   </si>
   <si>
     <t>751 Store Management (Rykec Puvyjo (10528834))</t>
@@ -418,58 +417,58 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF4A4A4A"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="6"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
       <family val="3"/>
-      <sz val="6"/>
-      <name val="Courier New"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF800000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -481,19 +480,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.5999938962981048"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499984740745262"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -524,8 +523,12 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -535,15 +538,25 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -554,14 +567,22 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -961,9 +982,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BP3"/>
-  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
@@ -1032,7 +1053,7 @@
     <col min="68" max="68" width="16.54296875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5" customHeight="1" spans="1:68" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="1" spans="1:68" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1238,49 +1259,45 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="E2" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="F2" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="G2" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="H2" s="18" t="s">
         <v>70</v>
-      </c>
-      <c r="G2" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="H2" s="18" t="s">
-        <v>72</v>
       </c>
       <c r="I2" s="19">
         <v>25041111</v>
       </c>
       <c r="J2" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="K2" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="L2" s="20">
+        <f t="shared" ref="L2" ca="1" si="0">TODAY()-31</f>
+        <v>45829</v>
+      </c>
+      <c r="M2" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="N2" s="21" t="s">
         <v>73</v>
-      </c>
-      <c r="K2" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="L2" s="20">
-        <f t="shared" ref="L2" si="0">TODAY()-31</f>
-        <v>45796</v>
-      </c>
-      <c r="M2" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="N2" s="21" t="s">
-        <v>75</v>
       </c>
       <c r="O2" s="19">
         <v>38</v>
@@ -1289,44 +1306,44 @@
         <v>1000</v>
       </c>
       <c r="Q2" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="R2" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="S2" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="T2" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="R2" s="19" t="s">
+      <c r="U2" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="S2" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="T2" s="22" t="s">
+      <c r="V2" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="W2" s="24">
+        <f t="shared" ref="W2" ca="1" si="1">L2</f>
+        <v>45829</v>
+      </c>
+      <c r="X2" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="U2" s="23" t="s">
+      <c r="Y2" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="V2" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="W2" s="24">
-        <f t="shared" ref="W2" si="1">L2</f>
-        <v>45796</v>
-      </c>
-      <c r="X2" s="19" t="s">
+      <c r="Z2" t="s">
         <v>80</v>
       </c>
-      <c r="Y2" s="25" t="s">
+      <c r="AA2" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AB2" t="s">
         <v>82</v>
       </c>
-      <c r="AA2" s="26" t="s">
+      <c r="AC2" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>84</v>
-      </c>
-      <c r="AC2" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="AD2" s="1" t="s">
         <v>52</v>
@@ -1335,162 +1352,158 @@
         <v>35</v>
       </c>
       <c r="AF2" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AH2" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AI2" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="AH2" s="20" t="s">
+      <c r="AJ2" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="AI2" s="19" t="s">
+      <c r="AK2" t="s">
         <v>89</v>
       </c>
-      <c r="AJ2" s="19" t="s">
+      <c r="AL2" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM2" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AN2" s="30">
+        <f t="array" aca="1" ref="AN2:AN3" ca="1">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
+        <v>87889516236</v>
+      </c>
+      <c r="AO2" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="AL2" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="AM2" s="29" t="s">
+      <c r="AP2" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="AN2" s="30">
-        <f t="array" ref="AN2:AN3">_xlfn.RANDARRAY(2,1,12345678901,99999999999,TRUE)</f>
-        <v>32523314551</v>
-      </c>
-      <c r="AO2" s="15" t="s">
+      <c r="AQ2" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="AP2" s="21" t="s">
+      <c r="AR2" s="20" t="str">
+        <f>AH2</f>
+        <v>N/A</v>
+      </c>
+      <c r="AS2" t="s">
         <v>94</v>
-      </c>
-      <c r="AQ2" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="AR2" s="20">
-        <f>AH2</f>
-        <v>NaN</v>
-      </c>
-      <c r="AS2" t="s">
-        <v>96</v>
       </c>
       <c r="AT2" s="31">
         <v>35591</v>
       </c>
       <c r="AU2" s="32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="AV2" s="29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="AW2" s="32" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="AX2" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="AY2" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="AZ2" s="32" t="s">
         <v>97</v>
       </c>
-      <c r="AY2" s="33" t="s">
+      <c r="BA2" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="BB2" t="s">
         <v>98</v>
       </c>
-      <c r="AZ2" s="32" t="s">
+      <c r="BC2" t="s">
         <v>99</v>
       </c>
-      <c r="BA2" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="BB2" t="s">
+      <c r="BD2" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BE2" s="29" t="s">
         <v>101</v>
       </c>
-      <c r="BD2" s="15" t="s">
+      <c r="BF2" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="BE2" s="29" t="s">
+      <c r="BG2" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="BF2" s="34" t="s">
+      <c r="BH2" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="BG2" s="29" t="s">
+      <c r="BI2" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="BH2" s="29" t="s">
+      <c r="BJ2" s="32" t="s">
         <v>106</v>
       </c>
-      <c r="BI2" s="29" t="s">
+      <c r="BK2" s="32" t="s">
         <v>107</v>
       </c>
-      <c r="BJ2" s="32" t="s">
+      <c r="BL2" s="32" t="s">
         <v>108</v>
       </c>
-      <c r="BK2" s="32" t="s">
+      <c r="BM2" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="BL2" s="32" t="s">
+      <c r="BN2" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="BM2" s="32" t="s">
+      <c r="BO2" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="BN2" s="32" t="s">
+      <c r="BP2" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="BO2" s="19" t="s">
+    </row>
+    <row r="3" spans="1:68" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="BP2" s="35" t="s">
+      <c r="B3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="14" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="3" ht="15.65" customHeight="1" spans="1:68" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="E3" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="G3" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="H3" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>119</v>
-      </c>
-      <c r="G3" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="H3" s="18" t="s">
-        <v>121</v>
       </c>
       <c r="I3" s="19">
         <v>25041111</v>
       </c>
       <c r="J3" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="L3" s="20">
+        <f t="shared" ref="L3" ca="1" si="2">TODAY()-31</f>
+        <v>45829</v>
+      </c>
+      <c r="M3" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="N3" s="21" t="s">
         <v>73</v>
-      </c>
-      <c r="K3" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="L3" s="20">
-        <f t="shared" ref="L3" si="2">TODAY()-31</f>
-        <v>45796</v>
-      </c>
-      <c r="M3" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="N3" s="21" t="s">
-        <v>75</v>
       </c>
       <c r="O3" s="19">
         <v>38</v>
@@ -1499,44 +1512,44 @@
         <v>1000</v>
       </c>
       <c r="Q3" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="R3" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="S3" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="T3" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="R3" s="19" t="s">
+      <c r="U3" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="S3" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="T3" s="22" t="s">
+      <c r="V3" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="W3" s="24">
+        <f t="shared" ref="W3" ca="1" si="3">L3</f>
+        <v>45829</v>
+      </c>
+      <c r="X3" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="U3" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="V3" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="W3" s="24">
-        <f t="shared" ref="W3" si="3">L3</f>
-        <v>45796</v>
-      </c>
-      <c r="X3" s="19" t="s">
-        <v>80</v>
-      </c>
       <c r="Y3" s="25" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="Z3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="AA3" s="26" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="AB3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="AC3" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>52</v>
@@ -1545,149 +1558,132 @@
         <v>35</v>
       </c>
       <c r="AF3" s="15" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="AG3" t="s">
+        <v>85</v>
+      </c>
+      <c r="AH3" s="20">
+        <f ca="1">TODAY()+365</f>
+        <v>46225</v>
+      </c>
+      <c r="AI3" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="AH3" s="20">
-        <f>TODAY()+365</f>
-        <v>46192</v>
-      </c>
-      <c r="AI3" s="19" t="s">
-        <v>89</v>
-      </c>
       <c r="AJ3" s="19" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="AK3" s="1">
         <v>251</v>
       </c>
       <c r="AL3" s="29" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="AM3" s="29" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AN3" s="30">
-        <v>96321136803</v>
+        <f ca="1"/>
+        <v>12636349194</v>
       </c>
       <c r="AO3" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="AP3" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="AQ3" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="AP3" s="21" t="s">
+      <c r="AR3" s="20">
+        <f t="shared" ref="AR3" ca="1" si="4">AH3</f>
+        <v>46225</v>
+      </c>
+      <c r="AS3" t="s">
         <v>123</v>
-      </c>
-      <c r="AQ3" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="AR3" s="20">
-        <f t="shared" ref="AR3" si="4">AH3</f>
-        <v>46192</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>127</v>
       </c>
       <c r="AT3" s="31">
         <v>35591</v>
       </c>
       <c r="AU3" s="32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="AV3" s="29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="AW3" s="32" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="AX3" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="AY3" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="AZ3" s="32" t="s">
         <v>97</v>
       </c>
-      <c r="AY3" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="AZ3" s="32" t="s">
-        <v>99</v>
-      </c>
       <c r="BA3" s="32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="BB3" s="36" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="BC3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="BD3" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="BE3" s="29" t="s">
+        <v>101</v>
+      </c>
+      <c r="BF3" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="BE3" s="29" t="s">
+      <c r="BG3" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="BF3" s="34" t="s">
+      <c r="BH3" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="BG3" s="29" t="s">
+      <c r="BI3" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="BH3" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="BI3" s="29" t="s">
-        <v>107</v>
-      </c>
       <c r="BJ3" s="32" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="BK3" s="32" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="BL3" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="BM3" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="BN3" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="BM3" s="32" t="s">
+      <c r="BO3" s="19" t="s">
         <v>111</v>
       </c>
-      <c r="BN3" s="32" t="s">
+      <c r="BP3" s="35" t="s">
         <v>112</v>
-      </c>
-      <c r="BO3" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="BP3" s="35" t="s">
-        <v>114</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ3">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX2:AX3">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BI2:BI3">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K3">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S2:S3">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V3">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X3">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ2:AQ3 X2:X3 V2:V3 S2:S3 K2:K3 BI2:BI3 AX2:AX3" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="U2" r:id="rId1"/>
-    <hyperlink ref="U3" r:id="rId2"/>
+    <hyperlink ref="U2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="U3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>